<commit_message>
feat: add error/duplicate notification dialog and improve responsive design for feeder scanning UI
</commit_message>
<xml_diff>
--- a/Intermittent Buzzer E-BOM-Rev-001_1 (1)1 (1).xlsx
+++ b/Intermittent Buzzer E-BOM-Rev-001_1 (1)1 (1).xlsx
@@ -13,7 +13,6 @@
   <externalReferences>
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
-    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName function="false" hidden="false" name="ALL" vbProcedure="false">#REF!</definedName>
@@ -34,7 +33,6 @@
     <definedName function="false" hidden="false" name="INTT" vbProcedure="false">#REF!</definedName>
     <definedName function="false" hidden="false" name="LAST8" vbProcedure="false">#REF!</definedName>
     <definedName function="false" hidden="false" name="MFG" vbProcedure="false">#REF!</definedName>
-    <definedName function="false" hidden="false" name="offset" vbProcedure="false">[4]Summary!$G$89</definedName>
     <definedName function="false" hidden="false" name="OH" vbProcedure="false">#REF!</definedName>
     <definedName function="false" hidden="false" name="ouc" vbProcedure="false">#REF!</definedName>
     <definedName function="false" hidden="false" name="OUTPUTFILENAME" vbProcedure="false">#REF!</definedName>
@@ -225,7 +223,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="90">
   <si>
     <t xml:space="preserve">BILL OF MATERIAL</t>
   </si>
@@ -252,6 +250,9 @@
   </si>
   <si>
     <t xml:space="preserve">SR NO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feeder Number </t>
   </si>
   <si>
     <t xml:space="preserve">Item Name</t>
@@ -296,6 +297,9 @@
     <t xml:space="preserve">Remarks</t>
   </si>
   <si>
+    <t xml:space="preserve">YSM-001</t>
+  </si>
+  <si>
     <t xml:space="preserve">CAPACITOR</t>
   </si>
   <si>
@@ -324,6 +328,9 @@
     <t xml:space="preserve">CC0603KRX7R9BB472</t>
   </si>
   <si>
+    <t xml:space="preserve">YSM-002</t>
+  </si>
+  <si>
     <t xml:space="preserve">RDSCAP0037</t>
   </si>
   <si>
@@ -339,6 +346,9 @@
     <t xml:space="preserve">CC0603KRX7R9BB104</t>
   </si>
   <si>
+    <t xml:space="preserve">YSM-003</t>
+  </si>
+  <si>
     <t xml:space="preserve">RESISTOR</t>
   </si>
   <si>
@@ -358,6 +368,9 @@
   </si>
   <si>
     <t xml:space="preserve">RC0603FR-074K7L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YSM-004</t>
   </si>
   <si>
     <t xml:space="preserve">RDSRES0502 YAGEO</t>
@@ -379,6 +392,9 @@
     <t xml:space="preserve">RC0805FR-07270KL</t>
   </si>
   <si>
+    <t xml:space="preserve">YSM-005</t>
+  </si>
+  <si>
     <t xml:space="preserve">RDSRES0235 YAGEO</t>
   </si>
   <si>
@@ -392,6 +408,9 @@
   </si>
   <si>
     <t xml:space="preserve"> RC0805JR-0710KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YSM-006</t>
   </si>
   <si>
     <t xml:space="preserve">RDSRES1109 ROYAL OHM</t>
@@ -410,6 +429,9 @@
 RC0603JR-072K7L</t>
   </si>
   <si>
+    <t xml:space="preserve">YSM-007</t>
+  </si>
+  <si>
     <t xml:space="preserve">RDSRES0985</t>
   </si>
   <si>
@@ -423,6 +445,9 @@
   </si>
   <si>
     <t xml:space="preserve"> RC0603FR-0710KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YSM-008</t>
   </si>
   <si>
     <t xml:space="preserve">555 IC</t>
@@ -1202,7 +1227,7 @@
     </fill>
     <fill>
       <patternFill patternType="darkGray">
-        <fgColor rgb="FF840032"/>
+        <fgColor rgb="FF7A0322"/>
         <bgColor rgb="FF333399"/>
       </patternFill>
     </fill>
@@ -1245,7 +1270,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF840032"/>
+        <bgColor rgb="FF7A0322"/>
       </patternFill>
     </fill>
     <fill>
@@ -1316,7 +1341,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF97CE06"/>
+        <fgColor rgb="FF96CF0C"/>
         <bgColor rgb="FFFFCC00"/>
       </patternFill>
     </fill>
@@ -1376,16 +1401,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="double">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </left>
       <right style="double">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </right>
       <top style="double">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </top>
       <bottom style="double">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1492,16 +1517,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </left>
       <right style="thin">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </right>
       <top style="thin">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF203620"/>
+        <color rgb="FF153815"/>
       </bottom>
       <diagonal/>
     </border>
@@ -4681,172 +4706,156 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="62" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="62" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="63" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="63" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="64" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="216" fontId="65" fillId="40" borderId="19" xfId="734" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="216" fontId="65" fillId="40" borderId="19" xfId="734" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="65" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="67" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="67" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="216" fontId="65" fillId="40" borderId="19" xfId="734" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="216" fontId="65" fillId="40" borderId="19" xfId="734" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="64" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="65" fillId="49" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="66" fillId="49" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="65" fillId="49" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="66" fillId="49" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="65" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="67" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="68" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="49" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="65" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="69" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="70" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="70" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="69" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="71" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="185" fontId="71" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="72" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="73" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="66" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="64" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="49" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="66" fillId="49" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="49" borderId="19" xfId="595" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="66" fillId="49" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="67" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="68" fillId="49" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="49" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="65" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="69" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="70" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="70" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="69" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="71" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="185" fontId="71" fillId="0" borderId="20" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="71" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="72" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="73" fillId="0" borderId="18" xfId="593" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="593" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5801,11 +5810,11 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF840032"/>
+      <rgbColor rgb="FF7A0322"/>
       <rgbColor rgb="FFB7DEE8"/>
       <rgbColor rgb="FFEBF1DE"/>
       <rgbColor rgb="FFB2B2B2"/>
-      <rgbColor rgb="FFFCD5B5"/>
+      <rgbColor rgb="FFF2DCDB"/>
       <rgbColor rgb="FFB9CDE5"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
@@ -5813,16 +5822,16 @@
       <rgbColor rgb="FFFF9F9F"/>
       <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFE0E0E0"/>
+      <rgbColor rgb="FFE6E0EC"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FFFDEADA"/>
-      <rgbColor rgb="FFCFCFCF"/>
+      <rgbColor rgb="FFFCD5B5"/>
       <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FFA6D9FF"/>
-      <rgbColor rgb="FFF2DCDB"/>
-      <rgbColor rgb="FFE6E0EC"/>
+      <rgbColor rgb="FFE0E0E0"/>
+      <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFCCC1DA"/>
       <rgbColor rgb="FFDCE6F2"/>
       <rgbColor rgb="FF00CCFF"/>
@@ -5835,7 +5844,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF97CE06"/>
+      <rgbColor rgb="FF96CF0C"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -5843,51 +5852,18 @@
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF001A6B"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FFC6EFCE"/>
+      <rgbColor rgb="FF153815"/>
       <rgbColor rgb="FFD7E4BD"/>
       <rgbColor rgb="FF9B4400"/>
       <rgbColor rgb="FFE6B9B8"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF203620"/>
+      <rgbColor rgb="FFCFCFCF"/>
     </indexedColors>
   </colors>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Data"/>
-      <sheetName val="Balance Sheet"/>
-      <sheetName val="Cash Flow"/>
-      <sheetName val="SENSITIVITY"/>
-      <sheetName val="Summary"/>
-      <sheetName val="Capital Forecast Detail"/>
-      <sheetName val="Balance_Sheet"/>
-      <sheetName val="Cash_Flow"/>
-      <sheetName val="21"/>
-      <sheetName val="Total Machine Cost"/>
-      <sheetName val="repeatative rejection"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -5940,7 +5916,7 @@
 </externalLink>
 </file>
 
-<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -6398,25 +6374,25 @@
     <tabColor rgb="FF92D050"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:O1048576"/>
+  <dimension ref="A1:P1048576"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="77.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="86.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="31.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="64.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="36.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="76.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="83.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="43.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="51.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="27.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="26.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="73.85"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="77.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="86.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="64.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="36.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="76.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="83.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="43.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="51.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="27.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="26.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="73.85"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6424,28 +6400,29 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3"/>
+      <c r="N1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="4"/>
       <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
+      <c r="E2" s="2"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -6453,18 +6430,19 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="3"/>
+      <c r="N2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="4"/>
       <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="2"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -6472,11 +6450,12 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3"/>
+      <c r="N3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="4"/>
       <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
@@ -6489,15 +6468,16 @@
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="4"/>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="83.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -6510,36 +6490,37 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="4"/>
+      <c r="J5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H6" s="5" t="s">
@@ -6548,30 +6529,33 @@
       <c r="I6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="L6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="N6" s="6" t="s">
-        <v>17</v>
+      <c r="M6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="88.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="6"/>
-      <c r="D7" s="5"/>
+      <c r="D7" s="6"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -6583,495 +6567,529 @@
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
     </row>
     <row r="8" s="14" customFormat="true" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8" t="s">
+      <c r="B8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="C8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="12" t="s">
+      <c r="F8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="H8" s="13"/>
-      <c r="I8" s="12" t="s">
+      <c r="G8" s="11" t="s">
         <v>26</v>
       </c>
+      <c r="H8" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="13"/>
       <c r="J8" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="M8" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="N8" s="12"/>
       <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
     </row>
     <row r="9" s="14" customFormat="true" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="15" t="s">
+      <c r="B9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="13"/>
+      <c r="J9" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L9" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" s="13"/>
-      <c r="I9" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="J9" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="L9" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="M9" s="12"/>
+      <c r="M9" s="12" t="s">
+        <v>37</v>
+      </c>
       <c r="N9" s="12"/>
       <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>35</v>
+      <c r="B10" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H10" s="13"/>
-      <c r="I10" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="F10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="13"/>
       <c r="J10" s="12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="M10" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="M10" s="12" t="s">
+        <v>45</v>
+      </c>
       <c r="N10" s="12"/>
       <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="100.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="18" t="n">
+      <c r="B11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="F11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="I11" s="13"/>
+      <c r="J11" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="H11" s="13"/>
-      <c r="I11" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>46</v>
-      </c>
       <c r="K11" s="12" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M11" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="M11" s="12" t="s">
+        <v>52</v>
+      </c>
       <c r="N11" s="12"/>
       <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>35</v>
+      <c r="B12" s="6" t="s">
+        <v>53</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="16" t="s">
+      <c r="F12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="13"/>
-      <c r="I12" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="I12" s="13"/>
       <c r="J12" s="12" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="M12" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="M12" s="12" t="s">
+        <v>58</v>
+      </c>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
     </row>
-    <row r="13" s="28" customFormat="true" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="n">
+    <row r="13" s="24" customFormat="true" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B13" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="22" t="n">
+      <c r="B13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="G13" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="H13" s="26"/>
-      <c r="I13" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="J13" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="K13" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="L13" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="27"/>
+      <c r="F13" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13" s="22"/>
+      <c r="J13" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L13" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="M13" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21"/>
+      <c r="P13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>35</v>
+      <c r="B14" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="H14" s="13"/>
-      <c r="I14" s="12" t="s">
-        <v>39</v>
-      </c>
+      <c r="F14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="13"/>
       <c r="J14" s="12" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="M14" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="M14" s="12" t="s">
+        <v>70</v>
+      </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>63</v>
+      <c r="B15" s="6" t="s">
+        <v>71</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="H15" s="13"/>
-      <c r="I15" s="12" t="s">
-        <v>68</v>
-      </c>
+      <c r="F15" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="13"/>
       <c r="J15" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="K15" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>75</v>
+      </c>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
       <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D16" s="9" t="n">
+      <c r="B16" s="6"/>
+      <c r="C16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="G16" s="12"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="12"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="12"/>
+      <c r="I16" s="13"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
       <c r="L16" s="12"/>
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="97.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="29"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="29"/>
-      <c r="N17" s="29"/>
-      <c r="O17" s="29"/>
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
     </row>
-    <row r="18" s="33" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="31" t="s">
-        <v>77</v>
-      </c>
-      <c r="M18" s="31"/>
-      <c r="N18" s="31"/>
-      <c r="O18" s="31"/>
+    <row r="18" s="29" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
     </row>
-    <row r="19" s="39" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="35"/>
-      <c r="L19" s="35"/>
-      <c r="M19" s="35"/>
-      <c r="N19" s="35"/>
-      <c r="O19" s="35"/>
+    <row r="19" s="35" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="31"/>
+      <c r="P19" s="31"/>
     </row>
-    <row r="20" s="39" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35"/>
-      <c r="N20" s="35"/>
-      <c r="O20" s="35"/>
+    <row r="20" s="35" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="31"/>
+      <c r="M20" s="31"/>
+      <c r="N20" s="31"/>
+      <c r="O20" s="31"/>
+      <c r="P20" s="31"/>
     </row>
-    <row r="21" s="39" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="35"/>
-      <c r="O21" s="35"/>
+    <row r="21" s="35" customFormat="true" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="30"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
+      <c r="M21" s="31"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="31"/>
     </row>
     <row r="22" customFormat="false" ht="72.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40" t="s">
-        <v>79</v>
-      </c>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="M22" s="40"/>
-      <c r="N22" s="40"/>
-      <c r="O22" s="40"/>
+      <c r="A22" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="36"/>
+      <c r="M22" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="N22" s="36"/>
+      <c r="O22" s="36"/>
+      <c r="P22" s="36"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="41"/>
-      <c r="B23" s="41"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="41"/>
-      <c r="K23" s="41"/>
-      <c r="L23" s="41"/>
-      <c r="M23" s="41"/>
-      <c r="N23" s="41"/>
-      <c r="O23" s="41"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
+      <c r="K23" s="37"/>
+      <c r="L23" s="37"/>
+      <c r="M23" s="37"/>
+      <c r="N23" s="37"/>
+      <c r="O23" s="37"/>
+      <c r="P23" s="37"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="41"/>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="41"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="41"/>
-      <c r="O24" s="41"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="37"/>
+      <c r="M24" s="37"/>
+      <c r="N24" s="37"/>
+      <c r="O24" s="37"/>
+      <c r="P24" s="37"/>
     </row>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -7084,16 +7102,16 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="A1:D3"/>
-    <mergeCell ref="E1:L3"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="M3:O3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="I4:O4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="I5:O5"/>
+  <mergeCells count="41">
+    <mergeCell ref="A1:E3"/>
+    <mergeCell ref="F1:M3"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="J4:P4"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="J5:P5"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
@@ -7109,22 +7127,23 @@
     <mergeCell ref="M6:M7"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="O6:O7"/>
-    <mergeCell ref="A17:O17"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="L19:O19"/>
-    <mergeCell ref="E20:H20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="F22:K22"/>
-    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="A17:P17"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="M18:P18"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:P19"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="M20:P20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="M21:P21"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="G22:L22"/>
+    <mergeCell ref="M22:P22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.1" right="0.1" top="0.1" bottom="0.1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>